<commit_message>
fix: GOP N/D (calcula Today/MTD desde GOP% Forecast), banco 340 días (fechas 2025→2026, de 340 a 35 días), GOP fallback en lector_drr para futuros DRR
</commit_message>
<xml_diff>
--- a/datos-referencia/extracto_banco.xlsx
+++ b/datos-referencia/extracto_banco.xlsx
@@ -225,18 +225,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD"/>
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -252,7 +244,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -260,30 +252,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -583,28 +557,28 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="2">
-        <v>45839</v>
+      <c r="A2" s="1">
+        <v>46144</v>
       </c>
       <c r="B2" t="s">
         <v>6</v>
@@ -623,8 +597,8 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="2">
-        <v>45839</v>
+      <c r="A3" s="1">
+        <v>46144</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
@@ -643,8 +617,8 @@
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="2">
-        <v>45840</v>
+      <c r="A4" s="1">
+        <v>46145</v>
       </c>
       <c r="B4" t="s">
         <v>8</v>
@@ -663,8 +637,8 @@
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="2">
-        <v>45841</v>
+      <c r="A5" s="1">
+        <v>46146</v>
       </c>
       <c r="B5" t="s">
         <v>9</v>
@@ -683,8 +657,8 @@
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="2">
-        <v>45842</v>
+      <c r="A6" s="1">
+        <v>46147</v>
       </c>
       <c r="B6" t="s">
         <v>10</v>
@@ -703,8 +677,8 @@
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="2">
-        <v>45843</v>
+      <c r="A7" s="1">
+        <v>46148</v>
       </c>
       <c r="B7" t="s">
         <v>11</v>
@@ -723,8 +697,8 @@
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="2">
-        <v>45843</v>
+      <c r="A8" s="1">
+        <v>46148</v>
       </c>
       <c r="B8" t="s">
         <v>12</v>
@@ -743,8 +717,8 @@
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="2">
-        <v>45844</v>
+      <c r="A9" s="1">
+        <v>46149</v>
       </c>
       <c r="B9" t="s">
         <v>13</v>
@@ -763,8 +737,8 @@
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="2">
-        <v>45845</v>
+      <c r="A10" s="1">
+        <v>46150</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
@@ -783,8 +757,8 @@
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="2">
-        <v>45846</v>
+      <c r="A11" s="1">
+        <v>46151</v>
       </c>
       <c r="B11" t="s">
         <v>15</v>
@@ -803,8 +777,8 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="2">
-        <v>45847</v>
+      <c r="A12" s="1">
+        <v>46152</v>
       </c>
       <c r="B12" t="s">
         <v>16</v>
@@ -823,8 +797,8 @@
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="2">
-        <v>45848</v>
+      <c r="A13" s="1">
+        <v>46153</v>
       </c>
       <c r="B13" t="s">
         <v>17</v>
@@ -843,8 +817,8 @@
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="2">
-        <v>45849</v>
+      <c r="A14" s="1">
+        <v>46154</v>
       </c>
       <c r="B14" t="s">
         <v>18</v>
@@ -863,8 +837,8 @@
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="2">
-        <v>45850</v>
+      <c r="A15" s="1">
+        <v>46155</v>
       </c>
       <c r="B15" t="s">
         <v>19</v>
@@ -883,8 +857,8 @@
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="2">
-        <v>45851</v>
+      <c r="A16" s="1">
+        <v>46156</v>
       </c>
       <c r="B16" t="s">
         <v>20</v>
@@ -903,8 +877,8 @@
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="2">
-        <v>45852</v>
+      <c r="A17" s="1">
+        <v>46157</v>
       </c>
       <c r="B17" t="s">
         <v>21</v>
@@ -923,8 +897,8 @@
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="2">
-        <v>45853</v>
+      <c r="A18" s="1">
+        <v>46158</v>
       </c>
       <c r="B18" t="s">
         <v>22</v>
@@ -943,8 +917,8 @@
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="2">
-        <v>45853</v>
+      <c r="A19" s="1">
+        <v>46158</v>
       </c>
       <c r="B19" t="s">
         <v>23</v>
@@ -963,8 +937,8 @@
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="2">
-        <v>45854</v>
+      <c r="A20" s="1">
+        <v>46159</v>
       </c>
       <c r="B20" t="s">
         <v>24</v>
@@ -983,8 +957,8 @@
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="2">
-        <v>45855</v>
+      <c r="A21" s="1">
+        <v>46160</v>
       </c>
       <c r="B21" t="s">
         <v>25</v>
@@ -1003,8 +977,8 @@
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="2">
-        <v>45856</v>
+      <c r="A22" s="1">
+        <v>46161</v>
       </c>
       <c r="B22" t="s">
         <v>26</v>
@@ -1023,8 +997,8 @@
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="2">
-        <v>45858</v>
+      <c r="A23" s="1">
+        <v>46163</v>
       </c>
       <c r="B23" t="s">
         <v>27</v>
@@ -1043,8 +1017,8 @@
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="2">
-        <v>45858</v>
+      <c r="A24" s="1">
+        <v>46163</v>
       </c>
       <c r="B24" t="s">
         <v>28</v>
@@ -1063,8 +1037,8 @@
       </c>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="2">
-        <v>45858</v>
+      <c r="A25" s="1">
+        <v>46163</v>
       </c>
       <c r="B25" t="s">
         <v>29</v>
@@ -1083,8 +1057,8 @@
       </c>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="2">
-        <v>45860</v>
+      <c r="A26" s="1">
+        <v>46165</v>
       </c>
       <c r="B26" t="s">
         <v>30</v>
@@ -1103,8 +1077,8 @@
       </c>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="2">
-        <v>45863</v>
+      <c r="A27" s="1">
+        <v>46168</v>
       </c>
       <c r="B27" t="s">
         <v>31</v>
@@ -1123,8 +1097,8 @@
       </c>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="2">
-        <v>45865</v>
+      <c r="A28" s="1">
+        <v>46170</v>
       </c>
       <c r="B28" t="s">
         <v>32</v>
@@ -1143,8 +1117,8 @@
       </c>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="2">
-        <v>45866</v>
+      <c r="A29" s="1">
+        <v>46171</v>
       </c>
       <c r="B29" t="s">
         <v>33</v>
@@ -1163,8 +1137,8 @@
       </c>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="2">
-        <v>45866</v>
+      <c r="A30" s="1">
+        <v>46171</v>
       </c>
       <c r="B30" t="s">
         <v>34</v>
@@ -1183,8 +1157,8 @@
       </c>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="2">
-        <v>45869</v>
+      <c r="A31" s="1">
+        <v>46174</v>
       </c>
       <c r="B31" t="s">
         <v>35</v>

</xml_diff>

<commit_message>
fix(demo): shift all demo dates from July 2025 → June 2026 (+335 days) — ventas F&B, mermas, inventario, pos_ordenes, pos_ventas, extracto_banco
</commit_message>
<xml_diff>
--- a/datos-referencia/extracto_banco.xlsx
+++ b/datos-referencia/extracto_banco.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="92">
   <si>
     <t>fecha</t>
   </si>
@@ -32,6 +32,78 @@
   </si>
   <si>
     <t>saldo</t>
+  </si>
+  <si>
+    <t>2027-04-02</t>
+  </si>
+  <si>
+    <t>2027-04-03</t>
+  </si>
+  <si>
+    <t>2027-04-04</t>
+  </si>
+  <si>
+    <t>2027-04-05</t>
+  </si>
+  <si>
+    <t>2027-04-06</t>
+  </si>
+  <si>
+    <t>2027-04-07</t>
+  </si>
+  <si>
+    <t>2027-04-08</t>
+  </si>
+  <si>
+    <t>2027-04-09</t>
+  </si>
+  <si>
+    <t>2027-04-10</t>
+  </si>
+  <si>
+    <t>2027-04-11</t>
+  </si>
+  <si>
+    <t>2027-04-12</t>
+  </si>
+  <si>
+    <t>2027-04-13</t>
+  </si>
+  <si>
+    <t>2027-04-14</t>
+  </si>
+  <si>
+    <t>2027-04-15</t>
+  </si>
+  <si>
+    <t>2027-04-16</t>
+  </si>
+  <si>
+    <t>2027-04-17</t>
+  </si>
+  <si>
+    <t>2027-04-18</t>
+  </si>
+  <si>
+    <t>2027-04-19</t>
+  </si>
+  <si>
+    <t>2027-04-21</t>
+  </si>
+  <si>
+    <t>2027-04-23</t>
+  </si>
+  <si>
+    <t>2027-04-26</t>
+  </si>
+  <si>
+    <t>2027-04-28</t>
+  </si>
+  <si>
+    <t>2027-04-29</t>
+  </si>
+  <si>
+    <t>2027-05-02</t>
   </si>
   <si>
     <t>TPV REDSYS - LIQUIDACION DIARIA 30/06</t>
@@ -224,9 +296,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -256,9 +325,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -577,600 +645,600 @@
       </c>
     </row>
     <row r="2" spans="1:6">
-      <c r="A2" s="1">
-        <v>46144</v>
+      <c r="A2" t="s">
+        <v>6</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="C2">
         <v>8920</v>
       </c>
       <c r="D2" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
+        <v>62</v>
       </c>
       <c r="F2">
         <v>133920</v>
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="1">
-        <v>46144</v>
+      <c r="A3" t="s">
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>7</v>
+        <v>31</v>
       </c>
       <c r="C3">
         <v>45</v>
       </c>
       <c r="D3" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E3" t="s">
-        <v>39</v>
+        <v>63</v>
       </c>
       <c r="F3">
         <v>133875</v>
       </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="1">
-        <v>46145</v>
+      <c r="A4" t="s">
+        <v>7</v>
       </c>
       <c r="B4" t="s">
-        <v>8</v>
+        <v>32</v>
       </c>
       <c r="C4">
         <v>12450</v>
       </c>
       <c r="D4" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E4" t="s">
-        <v>40</v>
+        <v>64</v>
       </c>
       <c r="F4">
         <v>146325</v>
       </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="1">
-        <v>46146</v>
+      <c r="A5" t="s">
+        <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>33</v>
       </c>
       <c r="C5">
         <v>2390</v>
       </c>
       <c r="D5" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E5" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="F5">
         <v>143935</v>
       </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="1">
-        <v>46147</v>
+      <c r="A6" t="s">
+        <v>9</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>34</v>
       </c>
       <c r="C6">
         <v>4850</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E6" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="F6">
         <v>148785</v>
       </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="1">
-        <v>46148</v>
+      <c r="A7" t="s">
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="C7">
         <v>2460</v>
       </c>
       <c r="D7" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E7" t="s">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="F7">
         <v>151245</v>
       </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="1">
-        <v>46148</v>
+      <c r="A8" t="s">
+        <v>10</v>
       </c>
       <c r="B8" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="C8">
         <v>1850</v>
       </c>
       <c r="D8" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E8" t="s">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="F8">
         <v>149395</v>
       </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="1">
-        <v>46149</v>
+      <c r="A9" t="s">
+        <v>11</v>
       </c>
       <c r="B9" t="s">
-        <v>13</v>
+        <v>37</v>
       </c>
       <c r="C9">
         <v>11340</v>
       </c>
       <c r="D9" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E9" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="F9">
         <v>160735</v>
       </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="1">
-        <v>46150</v>
+      <c r="A10" t="s">
+        <v>12</v>
       </c>
       <c r="B10" t="s">
-        <v>14</v>
+        <v>38</v>
       </c>
       <c r="C10">
         <v>18500</v>
       </c>
       <c r="D10" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E10" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="F10">
         <v>142235</v>
       </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="1">
-        <v>46151</v>
+      <c r="A11" t="s">
+        <v>13</v>
       </c>
       <c r="B11" t="s">
-        <v>15</v>
+        <v>39</v>
       </c>
       <c r="C11">
         <v>4200</v>
       </c>
       <c r="D11" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E11" t="s">
-        <v>47</v>
+        <v>71</v>
       </c>
       <c r="F11">
         <v>138035</v>
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="1">
-        <v>46152</v>
+      <c r="A12" t="s">
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="C12">
         <v>3450</v>
       </c>
       <c r="D12" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E12" t="s">
-        <v>48</v>
+        <v>72</v>
       </c>
       <c r="F12">
         <v>134585</v>
       </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="1">
-        <v>46153</v>
+      <c r="A13" t="s">
+        <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>41</v>
       </c>
       <c r="C13">
         <v>8300</v>
       </c>
       <c r="D13" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E13" t="s">
-        <v>49</v>
+        <v>73</v>
       </c>
       <c r="F13">
         <v>142885</v>
       </c>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="1">
-        <v>46154</v>
+      <c r="A14" t="s">
+        <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="C14">
         <v>4000</v>
       </c>
       <c r="D14" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E14" t="s">
-        <v>50</v>
+        <v>74</v>
       </c>
       <c r="F14">
         <v>146885</v>
       </c>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="1">
-        <v>46155</v>
+      <c r="A15" t="s">
+        <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>19</v>
+        <v>43</v>
       </c>
       <c r="C15">
         <v>1890</v>
       </c>
       <c r="D15" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E15" t="s">
-        <v>51</v>
+        <v>75</v>
       </c>
       <c r="F15">
         <v>144995</v>
       </c>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="1">
-        <v>46156</v>
+      <c r="A16" t="s">
+        <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="C16">
         <v>9650</v>
       </c>
       <c r="D16" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E16" t="s">
-        <v>52</v>
+        <v>76</v>
       </c>
       <c r="F16">
         <v>154645</v>
       </c>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="1">
-        <v>46157</v>
+      <c r="A17" t="s">
+        <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="C17">
         <v>2100</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E17" t="s">
-        <v>53</v>
+        <v>77</v>
       </c>
       <c r="F17">
         <v>152545</v>
       </c>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="1">
-        <v>46158</v>
+      <c r="A18" t="s">
+        <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
       <c r="C18">
         <v>6720</v>
       </c>
       <c r="D18" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E18" t="s">
-        <v>54</v>
+        <v>78</v>
       </c>
       <c r="F18">
         <v>159265</v>
       </c>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="1">
-        <v>46158</v>
+      <c r="A19" t="s">
+        <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="C19">
         <v>892.3</v>
       </c>
       <c r="D19" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E19" t="s">
-        <v>55</v>
+        <v>79</v>
       </c>
       <c r="F19">
         <v>158372.7</v>
       </c>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="1">
-        <v>46159</v>
+      <c r="A20" t="s">
+        <v>21</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>48</v>
       </c>
       <c r="C20">
         <v>4800</v>
       </c>
       <c r="D20" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E20" t="s">
-        <v>56</v>
+        <v>80</v>
       </c>
       <c r="F20">
         <v>153572.7</v>
       </c>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="1">
-        <v>46160</v>
+      <c r="A21" t="s">
+        <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="C21">
         <v>171000</v>
       </c>
       <c r="D21" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E21" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="F21">
         <v>-17427.3</v>
       </c>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="1">
-        <v>46161</v>
+      <c r="A22" t="s">
+        <v>23</v>
       </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>50</v>
       </c>
       <c r="C22">
         <v>3200</v>
       </c>
       <c r="D22" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E22" t="s">
-        <v>58</v>
+        <v>82</v>
       </c>
       <c r="F22">
         <v>-14227.3</v>
       </c>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="1">
-        <v>46163</v>
+      <c r="A23" t="s">
+        <v>24</v>
       </c>
       <c r="B23" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="C23">
         <v>12100</v>
       </c>
       <c r="D23" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E23" t="s">
-        <v>59</v>
+        <v>83</v>
       </c>
       <c r="F23">
         <v>-2127.3</v>
       </c>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="1">
-        <v>46163</v>
+      <c r="A24" t="s">
+        <v>24</v>
       </c>
       <c r="B24" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="C24">
         <v>8920</v>
       </c>
       <c r="D24" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E24" t="s">
-        <v>60</v>
+        <v>84</v>
       </c>
       <c r="F24">
         <v>-11047.3</v>
       </c>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="1">
-        <v>46163</v>
+      <c r="A25" t="s">
+        <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>29</v>
+        <v>53</v>
       </c>
       <c r="C25">
         <v>3400</v>
       </c>
       <c r="D25" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E25" t="s">
-        <v>61</v>
+        <v>85</v>
       </c>
       <c r="F25">
         <v>-14447.3</v>
       </c>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="1">
-        <v>46165</v>
+      <c r="A26" t="s">
+        <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>54</v>
       </c>
       <c r="C26">
         <v>340</v>
       </c>
       <c r="D26" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E26" t="s">
-        <v>62</v>
+        <v>86</v>
       </c>
       <c r="F26">
         <v>-14107.3</v>
       </c>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="1">
-        <v>46168</v>
+      <c r="A27" t="s">
+        <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>31</v>
+        <v>55</v>
       </c>
       <c r="C27">
         <v>1250</v>
       </c>
       <c r="D27" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E27" t="s">
-        <v>63</v>
+        <v>87</v>
       </c>
       <c r="F27">
         <v>-15357.3</v>
       </c>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="1">
-        <v>46170</v>
+      <c r="A28" t="s">
+        <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>32</v>
+        <v>56</v>
       </c>
       <c r="C28">
         <v>10800</v>
       </c>
       <c r="D28" t="s">
-        <v>36</v>
+        <v>60</v>
       </c>
       <c r="E28" t="s">
-        <v>64</v>
+        <v>88</v>
       </c>
       <c r="F28">
         <v>-4557.3</v>
       </c>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="1">
-        <v>46171</v>
+      <c r="A29" t="s">
+        <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>33</v>
+        <v>57</v>
       </c>
       <c r="C29">
         <v>42300</v>
       </c>
       <c r="D29" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E29" t="s">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="F29">
         <v>-46857.3</v>
       </c>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="1">
-        <v>46171</v>
+      <c r="A30" t="s">
+        <v>28</v>
       </c>
       <c r="B30" t="s">
-        <v>34</v>
+        <v>58</v>
       </c>
       <c r="C30">
         <v>14200</v>
       </c>
       <c r="D30" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E30" t="s">
-        <v>66</v>
+        <v>90</v>
       </c>
       <c r="F30">
         <v>-61057.3</v>
       </c>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="1">
-        <v>46174</v>
+      <c r="A31" t="s">
+        <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>35</v>
+        <v>59</v>
       </c>
       <c r="C31">
         <v>128.5</v>
       </c>
       <c r="D31" t="s">
-        <v>37</v>
+        <v>61</v>
       </c>
       <c r="E31" t="s">
-        <v>67</v>
+        <v>91</v>
       </c>
       <c r="F31">
         <v>-61185.8</v>

</xml_diff>

<commit_message>
feat(phase1): DRR GOP fix + Budget col; banco dates May 2026; admin panel hotel registration form + API; AR Real emit invoice modal + /api/ar_real/emitir_factura; 404/500 branded error pages; login demo button; Y favicon; mobile CSS 768px breakpoint; Calipolis sparklines+trends API; email HTML professional template
</commit_message>
<xml_diff>
--- a/datos-referencia/extracto_banco.xlsx
+++ b/datos-referencia/extracto_banco.xlsx
@@ -34,76 +34,76 @@
     <t>saldo</t>
   </si>
   <si>
-    <t>2027-04-02</t>
-  </si>
-  <si>
-    <t>2027-04-03</t>
-  </si>
-  <si>
-    <t>2027-04-04</t>
-  </si>
-  <si>
-    <t>2027-04-05</t>
-  </si>
-  <si>
-    <t>2027-04-06</t>
-  </si>
-  <si>
-    <t>2027-04-07</t>
-  </si>
-  <si>
-    <t>2027-04-08</t>
-  </si>
-  <si>
-    <t>2027-04-09</t>
-  </si>
-  <si>
-    <t>2027-04-10</t>
-  </si>
-  <si>
-    <t>2027-04-11</t>
-  </si>
-  <si>
-    <t>2027-04-12</t>
-  </si>
-  <si>
-    <t>2027-04-13</t>
-  </si>
-  <si>
-    <t>2027-04-14</t>
-  </si>
-  <si>
-    <t>2027-04-15</t>
-  </si>
-  <si>
-    <t>2027-04-16</t>
-  </si>
-  <si>
-    <t>2027-04-17</t>
-  </si>
-  <si>
-    <t>2027-04-18</t>
-  </si>
-  <si>
-    <t>2027-04-19</t>
-  </si>
-  <si>
-    <t>2027-04-21</t>
-  </si>
-  <si>
-    <t>2027-04-23</t>
-  </si>
-  <si>
-    <t>2027-04-26</t>
-  </si>
-  <si>
-    <t>2027-04-28</t>
-  </si>
-  <si>
-    <t>2027-04-29</t>
-  </si>
-  <si>
-    <t>2027-05-02</t>
+    <t>2026-05-02</t>
+  </si>
+  <si>
+    <t>2026-05-03</t>
+  </si>
+  <si>
+    <t>2026-05-04</t>
+  </si>
+  <si>
+    <t>2026-05-05</t>
+  </si>
+  <si>
+    <t>2026-05-06</t>
+  </si>
+  <si>
+    <t>2026-05-07</t>
+  </si>
+  <si>
+    <t>2026-05-08</t>
+  </si>
+  <si>
+    <t>2026-05-09</t>
+  </si>
+  <si>
+    <t>2026-05-10</t>
+  </si>
+  <si>
+    <t>2026-05-11</t>
+  </si>
+  <si>
+    <t>2026-05-12</t>
+  </si>
+  <si>
+    <t>2026-05-13</t>
+  </si>
+  <si>
+    <t>2026-05-14</t>
+  </si>
+  <si>
+    <t>2026-05-15</t>
+  </si>
+  <si>
+    <t>2026-05-16</t>
+  </si>
+  <si>
+    <t>2026-05-17</t>
+  </si>
+  <si>
+    <t>2026-05-18</t>
+  </si>
+  <si>
+    <t>2026-05-19</t>
+  </si>
+  <si>
+    <t>2026-05-21</t>
+  </si>
+  <si>
+    <t>2026-05-23</t>
+  </si>
+  <si>
+    <t>2026-05-26</t>
+  </si>
+  <si>
+    <t>2026-05-28</t>
+  </si>
+  <si>
+    <t>2026-05-29</t>
+  </si>
+  <si>
+    <t>2026-06-01</t>
   </si>
   <si>
     <t>TPV REDSYS - LIQUIDACION DIARIA 30/06</t>

</xml_diff>